<commit_message>
[stanley] latest version of lab6
</commit_message>
<xml_diff>
--- a/Labs/Lab6/DataAverage/200cm_average_data.xlsx
+++ b/Labs/Lab6/DataAverage/200cm_average_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B121"/>
+  <dimension ref="A1:B92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,122 +450,122 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B3" t="n">
-        <v>169.26</v>
+        <v>196.33</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B4" t="n">
-        <v>74.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B5" t="n">
-        <v>93.44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B6" t="n">
-        <v>283.84</v>
+        <v>225.59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>122.67</v>
+        <v>130</v>
       </c>
       <c r="B7" t="n">
-        <v>197.85</v>
+        <v>288.59</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>122.33</v>
+        <v>129</v>
       </c>
       <c r="B8" t="n">
-        <v>91.09</v>
+        <v>126.38</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B9" t="n">
-        <v>164.55</v>
+        <v>192.29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>121.67</v>
+        <v>127</v>
       </c>
       <c r="B10" t="n">
-        <v>196.47</v>
+        <v>143.52</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>121.33</v>
+        <v>126</v>
       </c>
       <c r="B11" t="n">
-        <v>217.66</v>
+        <v>209.81</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B12" t="n">
-        <v>147.67</v>
+        <v>233.31</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>120.67</v>
+        <v>124</v>
       </c>
       <c r="B13" t="n">
-        <v>74.51000000000001</v>
+        <v>146.99</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>120.33</v>
+        <v>123</v>
       </c>
       <c r="B14" t="n">
-        <v>146.3</v>
+        <v>129.71</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B15" t="n">
-        <v>190.25</v>
+        <v>124.78</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>119.67</v>
+        <v>121</v>
       </c>
       <c r="B16" t="n">
-        <v>198.78</v>
+        <v>173.28</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>119.33</v>
+        <v>120</v>
       </c>
       <c r="B17" t="n">
-        <v>198.6</v>
+        <v>194.47</v>
       </c>
     </row>
     <row r="18">
@@ -573,831 +573,599 @@
         <v>119</v>
       </c>
       <c r="B18" t="n">
-        <v>111.62</v>
+        <v>198.92</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>118.67</v>
+        <v>118</v>
       </c>
       <c r="B19" t="n">
-        <v>126.45</v>
+        <v>116.84</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>118.33</v>
+        <v>117</v>
       </c>
       <c r="B20" t="n">
-        <v>184.32</v>
+        <v>166.97</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B21" t="n">
-        <v>198.52</v>
+        <v>162.84</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>117.67</v>
+        <v>115</v>
       </c>
       <c r="B22" t="n">
-        <v>198.54</v>
+        <v>188.49</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>117.33</v>
+        <v>114</v>
       </c>
       <c r="B23" t="n">
-        <v>102.17</v>
+        <v>198.21</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B24" t="n">
-        <v>111.98</v>
+        <v>105.96</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>116.67</v>
+        <v>112</v>
       </c>
       <c r="B25" t="n">
-        <v>172.94</v>
+        <v>156.87</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>116.33</v>
+        <v>111</v>
       </c>
       <c r="B26" t="n">
-        <v>211.78</v>
+        <v>153.98</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B27" t="n">
-        <v>234.05</v>
+        <v>182.07</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>115.67</v>
+        <v>109</v>
       </c>
       <c r="B28" t="n">
-        <v>97.06</v>
+        <v>197.8</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>115.33</v>
+        <v>108</v>
       </c>
       <c r="B29" t="n">
-        <v>92.08</v>
+        <v>95.15000000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="B30" t="n">
-        <v>165.35</v>
+        <v>143.87</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>114.67</v>
+        <v>106</v>
       </c>
       <c r="B31" t="n">
-        <v>208.51</v>
+        <v>138.45</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>113.67</v>
+        <v>105</v>
       </c>
       <c r="B32" t="n">
-        <v>131.52</v>
+        <v>173.82</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>112.67</v>
+        <v>104</v>
       </c>
       <c r="B33" t="n">
-        <v>79.83</v>
+        <v>197.35</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>111.67</v>
+        <v>103</v>
       </c>
       <c r="B34" t="n">
-        <v>51.85</v>
+        <v>142.59</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>110.67</v>
+        <v>102</v>
       </c>
       <c r="B35" t="n">
-        <v>173.58</v>
+        <v>127.52</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>109.67</v>
+        <v>101</v>
       </c>
       <c r="B36" t="n">
-        <v>223.65</v>
+        <v>117.83</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>108.67</v>
+        <v>100</v>
       </c>
       <c r="B37" t="n">
-        <v>145.07</v>
+        <v>172.22</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>107.67</v>
+        <v>99</v>
       </c>
       <c r="B38" t="n">
-        <v>128.14</v>
+        <v>189.35</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>106.67</v>
+        <v>98</v>
       </c>
       <c r="B39" t="n">
-        <v>123.55</v>
+        <v>143.1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>105.67</v>
+        <v>97</v>
       </c>
       <c r="B40" t="n">
-        <v>188.4</v>
+        <v>140.46</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>104.67</v>
+        <v>96</v>
       </c>
       <c r="B41" t="n">
-        <v>230.21</v>
+        <v>154.15</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>103.67</v>
+        <v>95</v>
       </c>
       <c r="B42" t="n">
-        <v>156.83</v>
+        <v>185.74</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>102.67</v>
+        <v>94</v>
       </c>
       <c r="B43" t="n">
-        <v>91.54000000000001</v>
+        <v>140.78</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>101.67</v>
+        <v>93</v>
       </c>
       <c r="B44" t="n">
-        <v>158.01</v>
+        <v>136.53</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>100.67</v>
+        <v>92</v>
       </c>
       <c r="B45" t="n">
-        <v>197.61</v>
+        <v>150.52</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>99.67</v>
+        <v>91</v>
       </c>
       <c r="B46" t="n">
-        <v>153.51</v>
+        <v>186.99</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>98.67</v>
+        <v>90</v>
       </c>
       <c r="B47" t="n">
-        <v>126.61</v>
+        <v>139.66</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>97.67</v>
+        <v>89</v>
       </c>
       <c r="B48" t="n">
-        <v>124.39</v>
+        <v>129.59</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>96.67</v>
+        <v>88</v>
       </c>
       <c r="B49" t="n">
-        <v>173.2</v>
+        <v>145.37</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>95.67</v>
+        <v>87</v>
       </c>
       <c r="B50" t="n">
-        <v>134.51</v>
+        <v>183.61</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>94.67</v>
+        <v>86</v>
       </c>
       <c r="B51" t="n">
-        <v>132</v>
+        <v>197.36</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>93.67</v>
+        <v>85</v>
       </c>
       <c r="B52" t="n">
-        <v>97.28</v>
+        <v>118.79</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>92.67</v>
+        <v>84</v>
       </c>
       <c r="B53" t="n">
-        <v>78.64</v>
+        <v>115.32</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>91.67</v>
+        <v>83</v>
       </c>
       <c r="B54" t="n">
-        <v>108.47</v>
+        <v>131.5</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>90.67</v>
+        <v>82</v>
       </c>
       <c r="B55" t="n">
-        <v>127.7</v>
+        <v>131.58</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>89.67</v>
+        <v>81</v>
       </c>
       <c r="B56" t="n">
-        <v>94.16</v>
+        <v>49.6</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>88.67</v>
+        <v>80</v>
       </c>
       <c r="B57" t="n">
-        <v>122.22</v>
+        <v>107.71</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>87.67</v>
+        <v>79</v>
       </c>
       <c r="B58" t="n">
-        <v>77.65000000000001</v>
+        <v>131.67</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>86.67</v>
+        <v>78</v>
       </c>
       <c r="B59" t="n">
-        <v>102.08</v>
+        <v>131.76</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>85.67</v>
+        <v>77</v>
       </c>
       <c r="B60" t="n">
-        <v>81.11</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>84.67</v>
+        <v>76</v>
       </c>
       <c r="B61" t="n">
-        <v>122.53</v>
+        <v>108.86</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>83.67</v>
+        <v>75</v>
       </c>
       <c r="B62" t="n">
-        <v>131.79</v>
+        <v>131.86</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>82.67</v>
+        <v>74</v>
       </c>
       <c r="B63" t="n">
-        <v>131.8</v>
+        <v>131.94</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>81.67</v>
+        <v>73</v>
       </c>
       <c r="B64" t="n">
-        <v>47.41</v>
+        <v>41.05</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>80.67</v>
+        <v>72</v>
       </c>
       <c r="B65" t="n">
-        <v>103.68</v>
+        <v>102.12</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>79.67</v>
+        <v>71</v>
       </c>
       <c r="B66" t="n">
-        <v>131.56</v>
+        <v>131.87</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>78.67</v>
+        <v>70</v>
       </c>
       <c r="B67" t="n">
-        <v>197.85</v>
+        <v>132.16</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>77.67</v>
+        <v>69</v>
       </c>
       <c r="B68" t="n">
-        <v>97.88</v>
+        <v>35.77</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>76.67</v>
+        <v>68</v>
       </c>
       <c r="B69" t="n">
-        <v>127.71</v>
+        <v>96.94</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>75.67</v>
+        <v>67</v>
       </c>
       <c r="B70" t="n">
-        <v>194.39</v>
+        <v>198</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>74.67</v>
+        <v>66</v>
       </c>
       <c r="B71" t="n">
-        <v>198.33</v>
+        <v>145.1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>73.67</v>
+        <v>65</v>
       </c>
       <c r="B72" t="n">
-        <v>94.39</v>
+        <v>76.54000000000001</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>72.67</v>
+        <v>64</v>
       </c>
       <c r="B73" t="n">
-        <v>117.03</v>
+        <v>157.47</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>71.67</v>
+        <v>63</v>
       </c>
       <c r="B74" t="n">
-        <v>193.46</v>
+        <v>198.64</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>70.67</v>
+        <v>62</v>
       </c>
       <c r="B75" t="n">
-        <v>198.71</v>
+        <v>142.79</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>69.67</v>
+        <v>61</v>
       </c>
       <c r="B76" t="n">
-        <v>148.7</v>
+        <v>123.68</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>68.67</v>
+        <v>60</v>
       </c>
       <c r="B77" t="n">
-        <v>101.57</v>
+        <v>150.86</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>67.67</v>
+        <v>59</v>
       </c>
       <c r="B78" t="n">
-        <v>193.08</v>
+        <v>196.09</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>66.67</v>
+        <v>58</v>
       </c>
       <c r="B79" t="n">
-        <v>223.11</v>
+        <v>200.07</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>65.67</v>
+        <v>57</v>
       </c>
       <c r="B80" t="n">
-        <v>86.72</v>
+        <v>156.39</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>64.67</v>
+        <v>56</v>
       </c>
       <c r="B81" t="n">
-        <v>108.33</v>
+        <v>139.66</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>63.67</v>
+        <v>55</v>
       </c>
       <c r="B82" t="n">
-        <v>186.79</v>
+        <v>219.25</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>62.67</v>
+        <v>54</v>
       </c>
       <c r="B83" t="n">
-        <v>251.81</v>
+        <v>191.89</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>61.67</v>
+        <v>53</v>
       </c>
       <c r="B84" t="n">
-        <v>191.99</v>
+        <v>161.32</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>60.67</v>
+        <v>52</v>
       </c>
       <c r="B85" t="n">
-        <v>88.20999999999999</v>
+        <v>130.55</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>59.67</v>
+        <v>51</v>
       </c>
       <c r="B86" t="n">
-        <v>181.53</v>
+        <v>214</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>58.67</v>
+        <v>50</v>
       </c>
       <c r="B87" t="n">
-        <v>248.26</v>
+        <v>294.48</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>57.67</v>
+        <v>49</v>
       </c>
       <c r="B88" t="n">
-        <v>191.01</v>
+        <v>147.47</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>56.67</v>
+        <v>48</v>
       </c>
       <c r="B89" t="n">
-        <v>87.61</v>
+        <v>127.42</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>61.5</v>
+        <v>47</v>
       </c>
       <c r="B90" t="n">
-        <v>179.81</v>
+        <v>204.24</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>60.5</v>
+        <v>46</v>
       </c>
       <c r="B91" t="n">
-        <v>237.22</v>
+        <v>289.42</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>59.5</v>
+        <v>45</v>
       </c>
       <c r="B92" t="n">
-        <v>185.68</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="n">
-        <v>73</v>
-      </c>
-      <c r="B93" t="n">
-        <v>56.54</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>72</v>
-      </c>
-      <c r="B94" t="n">
-        <v>145.48</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="n">
-        <v>71</v>
-      </c>
-      <c r="B95" t="n">
-        <v>198.01</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n">
-        <v>70</v>
-      </c>
-      <c r="B96" t="n">
-        <v>198.29</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n">
-        <v>69</v>
-      </c>
-      <c r="B97" t="n">
-        <v>49.92</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="n">
-        <v>68</v>
-      </c>
-      <c r="B98" t="n">
-        <v>133.56</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="n">
-        <v>67</v>
-      </c>
-      <c r="B99" t="n">
-        <v>197.72</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="n">
-        <v>66</v>
-      </c>
-      <c r="B100" t="n">
-        <v>198.34</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="n">
-        <v>65</v>
-      </c>
-      <c r="B101" t="n">
-        <v>44.11</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="n">
-        <v>64</v>
-      </c>
-      <c r="B102" t="n">
-        <v>137.92</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="n">
-        <v>63</v>
-      </c>
-      <c r="B103" t="n">
-        <v>197.45</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="n">
-        <v>62</v>
-      </c>
-      <c r="B104" t="n">
-        <v>199.33</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
-        <v>61</v>
-      </c>
-      <c r="B105" t="n">
-        <v>199.06</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="n">
-        <v>60</v>
-      </c>
-      <c r="B106" t="n">
-        <v>114.75</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
-        <v>59</v>
-      </c>
-      <c r="B107" t="n">
-        <v>188.29</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="n">
-        <v>58</v>
-      </c>
-      <c r="B108" t="n">
-        <v>200.64</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>57</v>
-      </c>
-      <c r="B109" t="n">
-        <v>343.81</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>56</v>
-      </c>
-      <c r="B110" t="n">
-        <v>82.94</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
-        <v>55</v>
-      </c>
-      <c r="B111" t="n">
-        <v>173.94</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>54</v>
-      </c>
-      <c r="B112" t="n">
-        <v>263.56</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>53</v>
-      </c>
-      <c r="B113" t="n">
-        <v>339.12</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>52</v>
-      </c>
-      <c r="B114" t="n">
-        <v>82.94</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>51</v>
-      </c>
-      <c r="B115" t="n">
-        <v>169.42</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="n">
-        <v>50</v>
-      </c>
-      <c r="B116" t="n">
-        <v>252.47</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="n">
-        <v>49</v>
-      </c>
-      <c r="B117" t="n">
-        <v>331.25</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="n">
-        <v>48</v>
-      </c>
-      <c r="B118" t="n">
-        <v>73.87</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="n">
-        <v>47</v>
-      </c>
-      <c r="B119" t="n">
-        <v>150.01</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="n">
-        <v>46</v>
-      </c>
-      <c r="B120" t="n">
-        <v>248.19</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="n">
-        <v>45</v>
-      </c>
-      <c r="B121" t="n">
-        <v>80.40000000000001</v>
+        <v>111.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>